<commit_message>
docs(control-plane): sync exact commit SHA into control-plane Excel workbooks
</commit_message>
<xml_diff>
--- a/docs/control-plane/03_REPOSITORY_REGISTRY.xlsx
+++ b/docs/control-plane/03_REPOSITORY_REGISTRY.xlsx
@@ -172,7 +172,7 @@
     <t>v1.1.2-online-production-hardened</t>
   </si>
   <si>
-    <t>HEAD</t>
+    <t>4f1c5da05d4b88705182c31a44c4d5b768dead50</t>
   </si>
   <si>
     <t>2026-09-05</t>
@@ -868,7 +868,7 @@
     <col min="9" max="9" width="18" customWidth="1"/>
     <col min="10" max="10" width="29" customWidth="1"/>
     <col min="11" max="12" width="37" customWidth="1"/>
-    <col min="13" max="13" width="24" customWidth="1"/>
+    <col min="13" max="13" width="44" customWidth="1"/>
     <col min="14" max="14" width="17" customWidth="1"/>
     <col min="15" max="15" width="16" customWidth="1"/>
     <col min="16" max="16" width="14" customWidth="1"/>
@@ -1189,7 +1189,7 @@
   <cols>
     <col min="1" max="1" width="24" customWidth="1"/>
     <col min="2" max="2" width="37" customWidth="1"/>
-    <col min="3" max="3" width="14" customWidth="1"/>
+    <col min="3" max="3" width="44" customWidth="1"/>
     <col min="4" max="4" width="23" customWidth="1"/>
     <col min="5" max="5" width="16" customWidth="1"/>
     <col min="6" max="7" width="14" customWidth="1"/>

</xml_diff>